<commit_message>
Foso: plan de corte en varillas comerciales de 6 m y uso de retales
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGm1Wo5xdbH6HEAejZfCqA
</commit_message>
<xml_diff>
--- a/cantidades/Foso_Ascensor_Acero_Concreto.xlsx
+++ b/cantidades/Foso_Ascensor_Acero_Concreto.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Parámetros" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Cartilla acero" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Concreto por elementos" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Plan de corte" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="128">
   <si>
     <t xml:space="preserve">FOSO DE ASCENSOR — RESUMEN DE ACERO Y CONCRETO</t>
   </si>
@@ -308,6 +309,105 @@
   </si>
   <si>
     <t xml:space="preserve">No dibujado en EST-02. Losa + 0.10 m por lado. Va aparte del concreto estructural.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLAN DE CORTE EN VARILLAS COMERCIALES DE 6.00 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cada fila es un patrón: cuántas varillas se cortan igual y qué piezas salen de cada una. 48 varillas #4 es el mínimo posible.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Longitud varilla (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patrón</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Varillas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pieza 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L1 (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pieza 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L2 (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pieza 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L3 (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pieza 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L4 (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usado por varilla (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retal c/u (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retal total (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uso del retal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3/M4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin retal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chatarra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Silletas para la parrilla superior de la losa (1 por retal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estacas de formaleta y de replanteo (3 de 0.50 m por retal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reserva para reponer una pieza mal cortada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total varillas #4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retal total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total varillas #3</t>
   </si>
 </sst>
 </file>
@@ -471,7 +571,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -569,6 +669,26 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1823,4 +1943,480 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:R13"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="52"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Q3" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="R3" s="26" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="G5" s="15" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="I5" s="15" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="27" t="n">
+        <f aca="false">SUM(E5,G5,I5,K5)</f>
+        <v>6</v>
+      </c>
+      <c r="M5" s="27" t="n">
+        <f aca="false">$R$3-L5</f>
+        <v>0</v>
+      </c>
+      <c r="N5" s="27" t="n">
+        <f aca="false">C5*M5</f>
+        <v>0</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="I6" s="15" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="27" t="n">
+        <f aca="false">SUM(E6,G6,I6,K6)</f>
+        <v>5.8</v>
+      </c>
+      <c r="M6" s="27" t="n">
+        <f aca="false">$R$3-L6</f>
+        <v>0.199999999999999</v>
+      </c>
+      <c r="N6" s="27" t="n">
+        <f aca="false">C6*M6</f>
+        <v>1.59999999999999</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="I7" s="15" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="27" t="n">
+        <f aca="false">SUM(E7,G7,I7,K7)</f>
+        <v>5.95</v>
+      </c>
+      <c r="M7" s="27" t="n">
+        <f aca="false">$R$3-L7</f>
+        <v>0.0499999999999998</v>
+      </c>
+      <c r="N7" s="27" t="n">
+        <f aca="false">C7*M7</f>
+        <v>0.349999999999999</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="27" t="n">
+        <f aca="false">SUM(E8,G8,I8,K8)</f>
+        <v>5.2</v>
+      </c>
+      <c r="M8" s="27" t="n">
+        <f aca="false">$R$3-L8</f>
+        <v>0.8</v>
+      </c>
+      <c r="N8" s="27" t="n">
+        <f aca="false">C8*M8</f>
+        <v>8</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="27" t="n">
+        <f aca="false">SUM(E9,G9,I9,K9)</f>
+        <v>4.4</v>
+      </c>
+      <c r="M9" s="27" t="n">
+        <f aca="false">$R$3-L9</f>
+        <v>1.6</v>
+      </c>
+      <c r="N9" s="27" t="n">
+        <f aca="false">C9*M9</f>
+        <v>12.8</v>
+      </c>
+      <c r="O9" s="4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="27" t="n">
+        <f aca="false">SUM(E10,G10,I10,K10)</f>
+        <v>1.75</v>
+      </c>
+      <c r="M10" s="27" t="n">
+        <f aca="false">$R$3-L10</f>
+        <v>4.25</v>
+      </c>
+      <c r="N10" s="27" t="n">
+        <f aca="false">C10*M10</f>
+        <v>4.25</v>
+      </c>
+      <c r="O10" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I11" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="K11" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L11" s="27" t="n">
+        <f aca="false">SUM(E11,G11,I11,K11)</f>
+        <v>6</v>
+      </c>
+      <c r="M11" s="27" t="n">
+        <f aca="false">$R$3-L11</f>
+        <v>0</v>
+      </c>
+      <c r="N11" s="27" t="n">
+        <f aca="false">C11*M11</f>
+        <v>0</v>
+      </c>
+      <c r="O11" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="B12" s="19"/>
+      <c r="C12" s="28" t="n">
+        <f aca="false">SUMIF(B5:B11,"#4",C5:C11)</f>
+        <v>48</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="19"/>
+      <c r="K12" s="19"/>
+      <c r="L12" s="19"/>
+      <c r="M12" s="19"/>
+      <c r="N12" s="29" t="n">
+        <f aca="false">SUMIF(B5:B11,"#4",N5:N11)</f>
+        <v>27</v>
+      </c>
+      <c r="O12" s="23" t="str">
+        <f aca="false">TEXT(C12*$R$3,"0.00")&amp;" ml comprados"</f>
+        <v>288.00 ml comprados</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="B13" s="19"/>
+      <c r="C13" s="28" t="n">
+        <f aca="false">SUMIF(B5:B11,"#3",C5:C11)</f>
+        <v>20</v>
+      </c>
+      <c r="D13" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="19"/>
+      <c r="L13" s="19"/>
+      <c r="M13" s="19"/>
+      <c r="N13" s="29" t="n">
+        <f aca="false">SUMIF(B5:B11,"#3",N5:N11)</f>
+        <v>0</v>
+      </c>
+      <c r="O13" s="23" t="str">
+        <f aca="false">TEXT(C13*$R$3,"0.00")&amp;" ml comprados"</f>
+        <v>120.00 ml comprados</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D12:M12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D13:M13"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Foso: silletas pasan a llamarse burritos (nombre usado en obra)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGm1Wo5xdbH6HEAejZfCqA
</commit_message>
<xml_diff>
--- a/cantidades/Foso_Ascensor_Acero_Concreto.xlsx
+++ b/cantidades/Foso_Ascensor_Acero_Concreto.xlsx
@@ -223,7 +223,7 @@
     <t xml:space="preserve">Fila 30 · Con gancho de 0.20 m</t>
   </si>
   <si>
-    <t xml:space="preserve">Silleta</t>
+    <t xml:space="preserve">Burrito</t>
   </si>
   <si>
     <t xml:space="preserve">Fila 31 · —</t>
@@ -385,7 +385,7 @@
     <t xml:space="preserve">M3/M4 — Muros, verticales</t>
   </si>
   <si>
-    <t xml:space="preserve">Silletas para la parrilla superior de la losa</t>
+    <t xml:space="preserve">Burritos para la parrilla superior de la losa</t>
   </si>
   <si>
     <t xml:space="preserve">PLAN DE CORTE — VARILLAS NUEVAS #4 DE 6.00 m (USANDO EL INVENTARIO)</t>
@@ -481,7 +481,7 @@
     <t xml:space="preserve">B: L2 2.60 + L1 2.20</t>
   </si>
   <si>
-    <t xml:space="preserve">Silletas para la parrilla superior (1 por retal)</t>
+    <t xml:space="preserve">Burritos para la parrilla superior (1 por retal)</t>
   </si>
   <si>
     <t xml:space="preserve">C: M1 2.10 + M1 2.10 + C1 1.80</t>
@@ -3154,7 +3154,7 @@
         <v>8</v>
       </c>
       <c r="F84" s="22" t="n">
-        <f aca="false">COUNTIF($E$33:$E$72,"Silleta")</f>
+        <f aca="false">COUNTIF($E$33:$E$72,"Burrito")</f>
         <v>8</v>
       </c>
       <c r="G84" s="22" t="n">

</xml_diff>

<commit_message>
Plan de corte: uso con elemento y lado del muro; M3 y M4 separados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGm1Wo5xdbH6HEAejZfCqA
</commit_message>
<xml_diff>
--- a/cantidades/Foso_Ascensor_Acero_Concreto.xlsx
+++ b/cantidades/Foso_Ascensor_Acero_Concreto.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="185">
   <si>
     <t xml:space="preserve">FOSO DE ASCENSOR — RESUMEN DE ACERO Y CONCRETO</t>
   </si>
@@ -223,13 +223,13 @@
     <t xml:space="preserve">Fila 30 · Con gancho de 0.20 m</t>
   </si>
   <si>
-    <t xml:space="preserve">Burrito</t>
+    <t xml:space="preserve">Burrito · Losa, parrilla superior</t>
   </si>
   <si>
     <t xml:space="preserve">Fila 31 · —</t>
   </si>
   <si>
-    <t xml:space="preserve">M3/M4</t>
+    <t xml:space="preserve">M3 · Muro lado X (1.30 m), vertical</t>
   </si>
   <si>
     <t xml:space="preserve">Fila 32 · —</t>
@@ -253,7 +253,7 @@
     <t xml:space="preserve">Fila 45 · Con patas de 0.20 m a cada lado</t>
   </si>
   <si>
-    <t xml:space="preserve">L2</t>
+    <t xml:space="preserve">L2 · Losa, sentido Y</t>
   </si>
   <si>
     <t xml:space="preserve">Fila 49 · Con ganchos a 180° de 20.4 cm</t>
@@ -265,7 +265,7 @@
     <t xml:space="preserve">Fila 54 · —</t>
   </si>
   <si>
-    <t xml:space="preserve">C1</t>
+    <t xml:space="preserve">C1 · Columna, longitudinal</t>
   </si>
   <si>
     <t xml:space="preserve">Fila 55 · —</t>
@@ -274,13 +274,13 @@
     <t xml:space="preserve">Fila 56 · Con pata de 20 cm a un lado</t>
   </si>
   <si>
-    <t xml:space="preserve">M1</t>
+    <t xml:space="preserve">M1 · Muro lado X (1.30 m), horizontal</t>
   </si>
   <si>
     <t xml:space="preserve">Fila 57 · —</t>
   </si>
   <si>
-    <t xml:space="preserve">L1</t>
+    <t xml:space="preserve">L1 · Losa, sentido X</t>
   </si>
   <si>
     <t xml:space="preserve">Fila 58 · —</t>
@@ -346,7 +346,7 @@
     <t xml:space="preserve">Fila 84 · —</t>
   </si>
   <si>
-    <t xml:space="preserve">M2</t>
+    <t xml:space="preserve">M2 · Muro lado Y (1.70 m), horizontal</t>
   </si>
   <si>
     <t xml:space="preserve">Fila 85 · —</t>
@@ -382,7 +382,7 @@
     <t xml:space="preserve">ML FALTANTES</t>
   </si>
   <si>
-    <t xml:space="preserve">M3/M4 — Muros, verticales</t>
+    <t xml:space="preserve">M4 · Muro lado Y (1.70 m), vertical</t>
   </si>
   <si>
     <t xml:space="preserve">Burritos para la parrilla superior de la losa</t>
@@ -409,46 +409,49 @@
     <t xml:space="preserve">VARILLAS</t>
   </si>
   <si>
-    <t xml:space="preserve">A: M2 2.50 + M3/M4 1.75 + M3/M4 1.75</t>
+    <t xml:space="preserve">A: M2 2.50 + M4 1.75 + M4 1.75</t>
   </si>
   <si>
     <t xml:space="preserve">Sin retal</t>
   </si>
   <si>
-    <t xml:space="preserve">B: M1 2.10 + M1 2.10 + C1 1.80</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C: L2 2.60 + L2 2.60</t>
+    <t xml:space="preserve">B: M2 2.50 + M3 1.75 + M3 1.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C: M1 2.10 + M1 2.10 + C1 1.80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D: L2 2.60 + L2 2.60</t>
   </si>
   <si>
     <t xml:space="preserve">Estacas de formaleta</t>
   </si>
   <si>
-    <t xml:space="preserve">D: L2 2.60 + L1 2.20</t>
+    <t xml:space="preserve">E: L2 2.60 + L1 2.20</t>
   </si>
   <si>
     <t xml:space="preserve">Estacas de formaleta y replanteo</t>
   </si>
   <si>
-    <t xml:space="preserve">E: L1 2.20 + M3/M4 1.75 + M3/M4 1.75</t>
+    <t xml:space="preserve">F: L1 2.20 + M3 1.75 + M3 1.75</t>
   </si>
   <si>
     <t xml:space="preserve">Chatarra</t>
   </si>
   <si>
-    <t xml:space="preserve">F: L1 2.20 + C1 1.80 + C1 1.80</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G: L2 2.60 + M3/M4 1.75</t>
+    <t xml:space="preserve">G: L1 2.20 + C1 1.80 + C1 1.80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H: L2 2.60 + M3 1.75</t>
   </si>
   <si>
     <t xml:space="preserve">Reserva para reponer una pieza</t>
   </si>
   <si>
-    <t xml:space="preserve">H: L2 2.60 + M1 2.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I: L1 2.20 + C1 1.80 + M3/M4 1.75</t>
+    <t xml:space="preserve">I: L2 2.60 + M1 2.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J: L1 2.20 + C1 1.80 + M3 1.75</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL VARILLAS</t>
@@ -457,7 +460,7 @@
     <t xml:space="preserve">PLAN DE CORTE — VARILLAS NUEVAS #3 DE 6.00 m</t>
   </si>
   <si>
-    <t xml:space="preserve">J: E1 1.50 + E1 1.50 + E1 1.50 + E1 1.50</t>
+    <t xml:space="preserve">K: E1 1.50 + E1 1.50 + E1 1.50 + E1 1.50</t>
   </si>
   <si>
     <t xml:space="preserve">RESUMEN DE COMPRA DE VARILLAS DE 6.00 m</t>
@@ -478,25 +481,25 @@
     <t xml:space="preserve">REFERENCIA — PLAN DE CORTE SIN USAR EL INVENTARIO (VARILLAS #4)</t>
   </si>
   <si>
-    <t xml:space="preserve">B: L2 2.60 + L1 2.20</t>
+    <t xml:space="preserve">C: L2 2.60 + L1 2.20</t>
   </si>
   <si>
     <t xml:space="preserve">Burritos para la parrilla superior (1 por retal)</t>
   </si>
   <si>
-    <t xml:space="preserve">C: M1 2.10 + M1 2.10 + C1 1.80</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D: L1 2.20 + C1 1.80 + C1 1.80</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E: L2 2.60 + M3/M4 1.75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F: L1 2.20 + C1 1.80 + M3/M4 1.75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G: L1 2.20 + L1 2.20</t>
+    <t xml:space="preserve">D: M1 2.10 + M1 2.10 + C1 1.80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E: L1 2.20 + C1 1.80 + C1 1.80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F: L2 2.60 + M3 1.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G: L1 2.20 + C1 1.80 + M3 1.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H: L1 2.20 + L1 2.20</t>
   </si>
   <si>
     <t xml:space="preserve">• Las patas y ganchos se figuran después de cortar cada pieza a su L de corte.</t>
@@ -1405,7 +1408,7 @@
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="11" t="n">
-        <f aca="false">ACERO!H99</f>
+        <f aca="false">ACERO!H101</f>
         <v>31</v>
       </c>
       <c r="D9" s="7" t="s">
@@ -1418,7 +1421,7 @@
       </c>
       <c r="B10" s="9"/>
       <c r="C10" s="11" t="n">
-        <f aca="false">ACERO!H105+1</f>
+        <f aca="false">ACERO!H107+1</f>
         <v>17</v>
       </c>
       <c r="D10" s="7" t="s">
@@ -1542,7 +1545,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="C2:J128"/>
+  <dimension ref="C2:J131"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="4"/>
@@ -1984,7 +1987,7 @@
       <c r="I32" s="18"/>
       <c r="J32" s="18"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="31" t="s">
         <v>65</v>
       </c>
@@ -2008,7 +2011,7 @@
       <c r="I33" s="35"/>
       <c r="J33" s="35"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="31" t="s">
         <v>67</v>
       </c>
@@ -2032,7 +2035,7 @@
       <c r="I34" s="35"/>
       <c r="J34" s="35"/>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C35" s="31" t="s">
         <v>69</v>
       </c>
@@ -2056,7 +2059,7 @@
       <c r="I35" s="35"/>
       <c r="J35" s="35"/>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C36" s="31" t="s">
         <v>70</v>
       </c>
@@ -2080,7 +2083,7 @@
       <c r="I36" s="35"/>
       <c r="J36" s="35"/>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C37" s="31" t="s">
         <v>71</v>
       </c>
@@ -2104,7 +2107,7 @@
       <c r="I37" s="35"/>
       <c r="J37" s="35"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C38" s="31" t="s">
         <v>72</v>
       </c>
@@ -2128,7 +2131,7 @@
       <c r="I38" s="35"/>
       <c r="J38" s="35"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C39" s="31" t="s">
         <v>73</v>
       </c>
@@ -2152,7 +2155,7 @@
       <c r="I39" s="35"/>
       <c r="J39" s="35"/>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C40" s="31" t="s">
         <v>74</v>
       </c>
@@ -2176,7 +2179,7 @@
       <c r="I40" s="35"/>
       <c r="J40" s="35"/>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C41" s="31" t="s">
         <v>75</v>
       </c>
@@ -2200,7 +2203,7 @@
       <c r="I41" s="35"/>
       <c r="J41" s="35"/>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C42" s="31" t="s">
         <v>77</v>
       </c>
@@ -2224,7 +2227,7 @@
       <c r="I42" s="35"/>
       <c r="J42" s="35"/>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C43" s="31" t="s">
         <v>78</v>
       </c>
@@ -2248,7 +2251,7 @@
       <c r="I43" s="35"/>
       <c r="J43" s="35"/>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C44" s="31" t="s">
         <v>79</v>
       </c>
@@ -2272,7 +2275,7 @@
       <c r="I44" s="35"/>
       <c r="J44" s="35"/>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C45" s="31" t="s">
         <v>81</v>
       </c>
@@ -2296,7 +2299,7 @@
       <c r="I45" s="35"/>
       <c r="J45" s="35"/>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C46" s="31" t="s">
         <v>82</v>
       </c>
@@ -2320,7 +2323,7 @@
       <c r="I46" s="35"/>
       <c r="J46" s="35"/>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C47" s="31" t="s">
         <v>84</v>
       </c>
@@ -2344,7 +2347,7 @@
       <c r="I47" s="35"/>
       <c r="J47" s="35"/>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C48" s="31" t="s">
         <v>86</v>
       </c>
@@ -2368,7 +2371,7 @@
       <c r="I48" s="35"/>
       <c r="J48" s="35"/>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C49" s="31" t="s">
         <v>87</v>
       </c>
@@ -2392,7 +2395,7 @@
       <c r="I49" s="35"/>
       <c r="J49" s="35"/>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C50" s="31" t="s">
         <v>88</v>
       </c>
@@ -2416,7 +2419,7 @@
       <c r="I50" s="35"/>
       <c r="J50" s="35"/>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C51" s="31" t="s">
         <v>89</v>
       </c>
@@ -2440,7 +2443,7 @@
       <c r="I51" s="35"/>
       <c r="J51" s="35"/>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C52" s="31" t="s">
         <v>90</v>
       </c>
@@ -2464,7 +2467,7 @@
       <c r="I52" s="35"/>
       <c r="J52" s="35"/>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C53" s="31" t="s">
         <v>91</v>
       </c>
@@ -2488,7 +2491,7 @@
       <c r="I53" s="35"/>
       <c r="J53" s="35"/>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C54" s="31" t="s">
         <v>92</v>
       </c>
@@ -2512,7 +2515,7 @@
       <c r="I54" s="35"/>
       <c r="J54" s="35"/>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C55" s="31" t="s">
         <v>93</v>
       </c>
@@ -2536,7 +2539,7 @@
       <c r="I55" s="35"/>
       <c r="J55" s="35"/>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C56" s="31" t="s">
         <v>94</v>
       </c>
@@ -2560,7 +2563,7 @@
       <c r="I56" s="35"/>
       <c r="J56" s="35"/>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C57" s="31" t="s">
         <v>95</v>
       </c>
@@ -2584,7 +2587,7 @@
       <c r="I57" s="35"/>
       <c r="J57" s="35"/>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C58" s="31" t="s">
         <v>96</v>
       </c>
@@ -2608,7 +2611,7 @@
       <c r="I58" s="35"/>
       <c r="J58" s="35"/>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C59" s="31" t="s">
         <v>97</v>
       </c>
@@ -2632,7 +2635,7 @@
       <c r="I59" s="35"/>
       <c r="J59" s="35"/>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C60" s="31" t="s">
         <v>98</v>
       </c>
@@ -2656,7 +2659,7 @@
       <c r="I60" s="35"/>
       <c r="J60" s="35"/>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C61" s="31" t="s">
         <v>99</v>
       </c>
@@ -2680,7 +2683,7 @@
       <c r="I61" s="35"/>
       <c r="J61" s="35"/>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C62" s="31" t="s">
         <v>100</v>
       </c>
@@ -2704,7 +2707,7 @@
       <c r="I62" s="35"/>
       <c r="J62" s="35"/>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C63" s="31" t="s">
         <v>101</v>
       </c>
@@ -2728,7 +2731,7 @@
       <c r="I63" s="35"/>
       <c r="J63" s="35"/>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C64" s="31" t="s">
         <v>102</v>
       </c>
@@ -2752,7 +2755,7 @@
       <c r="I64" s="35"/>
       <c r="J64" s="35"/>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C65" s="31" t="s">
         <v>103</v>
       </c>
@@ -2776,7 +2779,7 @@
       <c r="I65" s="35"/>
       <c r="J65" s="35"/>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C66" s="31" t="s">
         <v>104</v>
       </c>
@@ -2800,7 +2803,7 @@
       <c r="I66" s="35"/>
       <c r="J66" s="35"/>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C67" s="31" t="s">
         <v>105</v>
       </c>
@@ -2824,7 +2827,7 @@
       <c r="I67" s="35"/>
       <c r="J67" s="35"/>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C68" s="31" t="s">
         <v>106</v>
       </c>
@@ -2848,7 +2851,7 @@
       <c r="I68" s="35"/>
       <c r="J68" s="35"/>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C69" s="31" t="s">
         <v>108</v>
       </c>
@@ -2872,7 +2875,7 @@
       <c r="I69" s="35"/>
       <c r="J69" s="35"/>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C70" s="31" t="s">
         <v>109</v>
       </c>
@@ -2896,7 +2899,7 @@
       <c r="I70" s="35"/>
       <c r="J70" s="35"/>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C71" s="31" t="s">
         <v>110</v>
       </c>
@@ -2920,7 +2923,7 @@
       <c r="I71" s="35"/>
       <c r="J71" s="35"/>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C72" s="31" t="s">
         <v>111</v>
       </c>
@@ -2995,7 +2998,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C78" s="19" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="D78" s="24" t="n">
         <v>2.2</v>
@@ -3004,7 +3007,7 @@
         <v>22</v>
       </c>
       <c r="F78" s="22" t="n">
-        <f aca="false">COUNTIF($E$33:$E$72,"L1")</f>
+        <f aca="false">COUNTIF($E$33:$E$72,"L1 ·*")</f>
         <v>14</v>
       </c>
       <c r="G78" s="22" t="n">
@@ -3020,7 +3023,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C79" s="19" t="s">
-        <v>38</v>
+        <v>76</v>
       </c>
       <c r="D79" s="24" t="n">
         <v>2.6</v>
@@ -3029,7 +3032,7 @@
         <v>18</v>
       </c>
       <c r="F79" s="22" t="n">
-        <f aca="false">COUNTIF($E$33:$E$72,"L2")</f>
+        <f aca="false">COUNTIF($E$33:$E$72,"L2 ·*")</f>
         <v>5</v>
       </c>
       <c r="G79" s="22" t="n">
@@ -3045,7 +3048,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C80" s="19" t="s">
-        <v>40</v>
+        <v>83</v>
       </c>
       <c r="D80" s="24" t="n">
         <v>2.1</v>
@@ -3054,7 +3057,7 @@
         <v>14</v>
       </c>
       <c r="F80" s="22" t="n">
-        <f aca="false">COUNTIF($E$33:$E$72,"M1")</f>
+        <f aca="false">COUNTIF($E$33:$E$72,"M1 ·*")</f>
         <v>1</v>
       </c>
       <c r="G80" s="22" t="n">
@@ -3070,7 +3073,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C81" s="19" t="s">
-        <v>42</v>
+        <v>107</v>
       </c>
       <c r="D81" s="24" t="n">
         <v>2.5</v>
@@ -3079,7 +3082,7 @@
         <v>14</v>
       </c>
       <c r="F81" s="22" t="n">
-        <f aca="false">COUNTIF($E$33:$E$72,"M2")</f>
+        <f aca="false">COUNTIF($E$33:$E$72,"M2 ·*")</f>
         <v>3</v>
       </c>
       <c r="G81" s="22" t="n">
@@ -3095,168 +3098,168 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C82" s="19" t="s">
-        <v>119</v>
+        <v>68</v>
       </c>
       <c r="D82" s="24" t="n">
         <v>1.75</v>
       </c>
       <c r="E82" s="22" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="F82" s="22" t="n">
-        <f aca="false">COUNTIF($E$33:$E$72,"M3/M4")</f>
+        <f aca="false">COUNTIF($E$33:$E$72,"M3 ·*")</f>
         <v>4</v>
       </c>
       <c r="G82" s="22" t="n">
         <f aca="false">E82-F82</f>
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="H82" s="24" t="n">
         <f aca="false">G82*D82</f>
-        <v>49</v>
+        <v>17.5</v>
       </c>
       <c r="I82" s="24"/>
       <c r="J82" s="24"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C83" s="19" t="s">
-        <v>47</v>
+        <v>119</v>
       </c>
       <c r="D83" s="24" t="n">
-        <v>1.8</v>
+        <v>1.75</v>
       </c>
       <c r="E83" s="22" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F83" s="22" t="n">
-        <f aca="false">COUNTIF($E$33:$E$72,"C1")</f>
-        <v>5</v>
+        <f aca="false">COUNTIF($E$33:$E$72,"M4 ·*")</f>
+        <v>0</v>
       </c>
       <c r="G83" s="22" t="n">
         <f aca="false">E83-F83</f>
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="H83" s="24" t="n">
         <f aca="false">G83*D83</f>
-        <v>19.8</v>
+        <v>31.5</v>
       </c>
       <c r="I83" s="24"/>
       <c r="J83" s="24"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C84" s="19" t="s">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="D84" s="24" t="n">
-        <v>0.75</v>
+        <v>1.8</v>
       </c>
       <c r="E84" s="22" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F84" s="22" t="n">
-        <f aca="false">COUNTIF($E$33:$E$72,"Burrito")</f>
-        <v>8</v>
+        <f aca="false">COUNTIF($E$33:$E$72,"C1 ·*")</f>
+        <v>5</v>
       </c>
       <c r="G84" s="22" t="n">
         <f aca="false">E84-F84</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H84" s="24" t="n">
         <f aca="false">G84*D84</f>
-        <v>0</v>
+        <v>19.8</v>
       </c>
       <c r="I84" s="24"/>
       <c r="J84" s="24"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C85" s="25" t="s">
+      <c r="C85" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="D85" s="24" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E85" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="F85" s="22" t="n">
+        <f aca="false">COUNTIF($E$33:$E$72,"Burrito ·*")</f>
+        <v>8</v>
+      </c>
+      <c r="G85" s="22" t="n">
+        <f aca="false">E85-F85</f>
+        <v>0</v>
+      </c>
+      <c r="H85" s="24" t="n">
+        <f aca="false">G85*D85</f>
+        <v>0</v>
+      </c>
+      <c r="I85" s="24"/>
+      <c r="J85" s="24"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C86" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="D85" s="26"/>
-      <c r="E85" s="27" t="n">
-        <f aca="false">SUM(E78:E84)</f>
+      <c r="D86" s="26"/>
+      <c r="E86" s="27" t="n">
+        <f aca="false">SUM(E78:E85)</f>
         <v>124</v>
       </c>
-      <c r="F85" s="27" t="n">
-        <f aca="false">SUM(F78:F84)</f>
+      <c r="F86" s="27" t="n">
+        <f aca="false">SUM(F78:F85)</f>
         <v>40</v>
       </c>
-      <c r="G85" s="27" t="n">
-        <f aca="false">SUM(G78:G84)</f>
+      <c r="G86" s="27" t="n">
+        <f aca="false">SUM(G78:G85)</f>
         <v>84</v>
       </c>
-      <c r="H85" s="26" t="n">
-        <f aca="false">SUM(H78:H84)</f>
+      <c r="H86" s="26" t="n">
+        <f aca="false">SUM(H78:H85)</f>
         <v>175</v>
       </c>
-      <c r="I85" s="26"/>
-      <c r="J85" s="26"/>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C88" s="16" t="s">
+      <c r="I86" s="26"/>
+      <c r="J86" s="26"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C89" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="D88" s="16"/>
-      <c r="E88" s="16"/>
-      <c r="F88" s="16"/>
-      <c r="G88" s="16"/>
-      <c r="H88" s="16"/>
-      <c r="I88" s="16"/>
-      <c r="J88" s="16"/>
-    </row>
-    <row r="89" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C89" s="17" t="s">
+      <c r="D89" s="16"/>
+      <c r="E89" s="16"/>
+      <c r="F89" s="16"/>
+      <c r="G89" s="16"/>
+      <c r="H89" s="16"/>
+      <c r="I89" s="16"/>
+      <c r="J89" s="16"/>
+    </row>
+    <row r="90" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C90" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="D89" s="18" t="s">
+      <c r="D90" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="E89" s="18" t="s">
+      <c r="E90" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F89" s="18" t="s">
+      <c r="F90" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="G89" s="18" t="s">
+      <c r="G90" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H89" s="18" t="s">
+      <c r="H90" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I89" s="18"/>
-      <c r="J89" s="18"/>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C90" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="D90" s="24" t="n">
-        <f aca="false">2.5+1.75+1.75</f>
-        <v>6</v>
-      </c>
-      <c r="E90" s="24" t="n">
-        <f aca="false">6-D90</f>
-        <v>0</v>
-      </c>
-      <c r="F90" s="20" t="s">
-        <v>129</v>
-      </c>
-      <c r="G90" s="24" t="n">
-        <f aca="false">E90*H90</f>
-        <v>0</v>
-      </c>
-      <c r="H90" s="36" t="n">
-        <v>11</v>
-      </c>
-      <c r="I90" s="36"/>
-      <c r="J90" s="36"/>
+      <c r="I90" s="18"/>
+      <c r="J90" s="18"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C91" s="19" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D91" s="24" t="n">
-        <f aca="false">2.1+2.1+1.8</f>
+        <f aca="false">2.5+1.75+1.75</f>
         <v>6</v>
       </c>
       <c r="E91" s="24" t="n">
@@ -3271,442 +3274,442 @@
         <v>0</v>
       </c>
       <c r="H91" s="36" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I91" s="36"/>
       <c r="J91" s="36"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C92" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="D92" s="24" t="n">
+        <f aca="false">2.5+1.75+1.75</f>
+        <v>6</v>
+      </c>
+      <c r="E92" s="24" t="n">
+        <f aca="false">6-D92</f>
+        <v>0</v>
+      </c>
+      <c r="F92" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="G92" s="24" t="n">
+        <f aca="false">E92*H92</f>
+        <v>0</v>
+      </c>
+      <c r="H92" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="I92" s="36"/>
+      <c r="J92" s="36"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C93" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="D92" s="24" t="n">
+      <c r="D93" s="24" t="n">
+        <f aca="false">2.1+2.1+1.8</f>
+        <v>6</v>
+      </c>
+      <c r="E93" s="24" t="n">
+        <f aca="false">6-D93</f>
+        <v>0</v>
+      </c>
+      <c r="F93" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="G93" s="24" t="n">
+        <f aca="false">E93*H93</f>
+        <v>0</v>
+      </c>
+      <c r="H93" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="I93" s="36"/>
+      <c r="J93" s="36"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C94" s="19" t="s">
+        <v>132</v>
+      </c>
+      <c r="D94" s="24" t="n">
         <f aca="false">2.6+2.6</f>
         <v>5.2</v>
       </c>
-      <c r="E92" s="24" t="n">
-        <f aca="false">6-D92</f>
+      <c r="E94" s="24" t="n">
+        <f aca="false">6-D94</f>
         <v>0.8</v>
       </c>
-      <c r="F92" s="20" t="s">
-        <v>132</v>
-      </c>
-      <c r="G92" s="24" t="n">
-        <f aca="false">E92*H92</f>
+      <c r="F94" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="G94" s="24" t="n">
+        <f aca="false">E94*H94</f>
         <v>3.2</v>
       </c>
-      <c r="H92" s="36" t="n">
+      <c r="H94" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="I92" s="36"/>
-      <c r="J92" s="36"/>
-    </row>
-    <row r="93" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C93" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="D93" s="24" t="n">
+      <c r="I94" s="36"/>
+      <c r="J94" s="36"/>
+    </row>
+    <row r="95" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C95" s="19" t="s">
+        <v>134</v>
+      </c>
+      <c r="D95" s="24" t="n">
         <f aca="false">2.6+2.2</f>
         <v>4.8</v>
       </c>
-      <c r="E93" s="24" t="n">
-        <f aca="false">6-D93</f>
+      <c r="E95" s="24" t="n">
+        <f aca="false">6-D95</f>
         <v>1.2</v>
       </c>
-      <c r="F93" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="G93" s="24" t="n">
-        <f aca="false">E93*H93</f>
+      <c r="F95" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="G95" s="24" t="n">
+        <f aca="false">E95*H95</f>
         <v>3.6</v>
       </c>
-      <c r="H93" s="36" t="n">
+      <c r="H95" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="I93" s="36"/>
-      <c r="J93" s="36"/>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C94" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="D94" s="24" t="n">
+      <c r="I95" s="36"/>
+      <c r="J95" s="36"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C96" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="D96" s="24" t="n">
         <f aca="false">2.2+1.75+1.75</f>
         <v>5.7</v>
       </c>
-      <c r="E94" s="24" t="n">
-        <f aca="false">6-D94</f>
+      <c r="E96" s="24" t="n">
+        <f aca="false">6-D96</f>
         <v>0.3</v>
       </c>
-      <c r="F94" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="G94" s="24" t="n">
-        <f aca="false">E94*H94</f>
+      <c r="F96" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="G96" s="24" t="n">
+        <f aca="false">E96*H96</f>
         <v>0.6</v>
       </c>
-      <c r="H94" s="36" t="n">
+      <c r="H96" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="I94" s="36"/>
-      <c r="J94" s="36"/>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C95" s="19" t="s">
-        <v>137</v>
-      </c>
-      <c r="D95" s="24" t="n">
+      <c r="I96" s="36"/>
+      <c r="J96" s="36"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C97" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="D97" s="24" t="n">
         <f aca="false">2.2+1.8+1.8</f>
         <v>5.8</v>
       </c>
-      <c r="E95" s="24" t="n">
-        <f aca="false">6-D95</f>
+      <c r="E97" s="24" t="n">
+        <f aca="false">6-D97</f>
         <v>0.2</v>
       </c>
-      <c r="F95" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="G95" s="24" t="n">
-        <f aca="false">E95*H95</f>
+      <c r="F97" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="G97" s="24" t="n">
+        <f aca="false">E97*H97</f>
         <v>0.4</v>
       </c>
-      <c r="H95" s="36" t="n">
+      <c r="H97" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="I95" s="36"/>
-      <c r="J95" s="36"/>
-    </row>
-    <row r="96" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C96" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="D96" s="24" t="n">
+      <c r="I97" s="36"/>
+      <c r="J97" s="36"/>
+    </row>
+    <row r="98" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C98" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="D98" s="24" t="n">
         <f aca="false">2.6+1.75</f>
         <v>4.35</v>
       </c>
-      <c r="E96" s="24" t="n">
-        <f aca="false">6-D96</f>
+      <c r="E98" s="24" t="n">
+        <f aca="false">6-D98</f>
         <v>1.65</v>
       </c>
-      <c r="F96" s="20" t="s">
-        <v>139</v>
-      </c>
-      <c r="G96" s="24" t="n">
-        <f aca="false">E96*H96</f>
+      <c r="F98" s="20" t="s">
+        <v>140</v>
+      </c>
+      <c r="G98" s="24" t="n">
+        <f aca="false">E98*H98</f>
         <v>1.65</v>
       </c>
-      <c r="H96" s="36" t="n">
+      <c r="H98" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="I96" s="36"/>
-      <c r="J96" s="36"/>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C97" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="D97" s="24" t="n">
+      <c r="I98" s="36"/>
+      <c r="J98" s="36"/>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C99" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="D99" s="24" t="n">
         <f aca="false">2.6+2.1</f>
         <v>4.7</v>
       </c>
-      <c r="E97" s="24" t="n">
-        <f aca="false">6-D97</f>
+      <c r="E99" s="24" t="n">
+        <f aca="false">6-D99</f>
         <v>1.3</v>
       </c>
-      <c r="F97" s="20" t="s">
-        <v>132</v>
-      </c>
-      <c r="G97" s="24" t="n">
-        <f aca="false">E97*H97</f>
+      <c r="F99" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="G99" s="24" t="n">
+        <f aca="false">E99*H99</f>
         <v>1.3</v>
       </c>
-      <c r="H97" s="36" t="n">
+      <c r="H99" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="I97" s="36"/>
-      <c r="J97" s="36"/>
-    </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C98" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="D98" s="24" t="n">
+      <c r="I99" s="36"/>
+      <c r="J99" s="36"/>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C100" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="D100" s="24" t="n">
         <f aca="false">2.2+1.8+1.75</f>
         <v>5.75</v>
       </c>
-      <c r="E98" s="24" t="n">
-        <f aca="false">6-D98</f>
+      <c r="E100" s="24" t="n">
+        <f aca="false">6-D100</f>
         <v>0.25</v>
       </c>
-      <c r="F98" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="G98" s="24" t="n">
-        <f aca="false">E98*H98</f>
+      <c r="F100" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="G100" s="24" t="n">
+        <f aca="false">E100*H100</f>
         <v>0.25</v>
       </c>
-      <c r="H98" s="36" t="n">
+      <c r="H100" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="I98" s="36"/>
-      <c r="J98" s="36"/>
-    </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C99" s="25" t="s">
-        <v>142</v>
-      </c>
-      <c r="D99" s="26"/>
-      <c r="E99" s="26"/>
-      <c r="F99" s="26"/>
-      <c r="G99" s="26" t="n">
-        <f aca="false">SUM(G90:G98)</f>
+      <c r="I100" s="36"/>
+      <c r="J100" s="36"/>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C101" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="D101" s="26"/>
+      <c r="E101" s="26"/>
+      <c r="F101" s="26"/>
+      <c r="G101" s="26" t="n">
+        <f aca="false">SUM(G91:G100)</f>
         <v>11</v>
       </c>
-      <c r="H99" s="27" t="n">
-        <f aca="false">SUM(H90:H98)</f>
+      <c r="H101" s="27" t="n">
+        <f aca="false">SUM(H91:H100)</f>
         <v>31</v>
       </c>
-      <c r="I99" s="27"/>
-      <c r="J99" s="27"/>
-    </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C102" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="D102" s="16"/>
-      <c r="E102" s="16"/>
-      <c r="F102" s="16"/>
-      <c r="G102" s="16"/>
-      <c r="H102" s="16"/>
-      <c r="I102" s="16"/>
-      <c r="J102" s="16"/>
-    </row>
-    <row r="103" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C103" s="17" t="s">
+      <c r="I101" s="27"/>
+      <c r="J101" s="27"/>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C104" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="D104" s="16"/>
+      <c r="E104" s="16"/>
+      <c r="F104" s="16"/>
+      <c r="G104" s="16"/>
+      <c r="H104" s="16"/>
+      <c r="I104" s="16"/>
+      <c r="J104" s="16"/>
+    </row>
+    <row r="105" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C105" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="D103" s="18" t="s">
+      <c r="D105" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="E103" s="18" t="s">
+      <c r="E105" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F103" s="18" t="s">
+      <c r="F105" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="G103" s="18" t="s">
+      <c r="G105" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H103" s="18" t="s">
+      <c r="H105" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I103" s="18"/>
-      <c r="J103" s="18"/>
-    </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C104" s="19" t="s">
-        <v>144</v>
-      </c>
-      <c r="D104" s="24" t="n">
+      <c r="I105" s="18"/>
+      <c r="J105" s="18"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C106" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="D106" s="24" t="n">
         <f aca="false">1.5+1.5+1.5+1.5</f>
         <v>6</v>
       </c>
-      <c r="E104" s="24" t="n">
-        <f aca="false">6-D104</f>
+      <c r="E106" s="24" t="n">
+        <f aca="false">6-D106</f>
         <v>0</v>
       </c>
-      <c r="F104" s="20" t="s">
+      <c r="F106" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="G104" s="24" t="n">
-        <f aca="false">E104*H104</f>
+      <c r="G106" s="24" t="n">
+        <f aca="false">E106*H106</f>
         <v>0</v>
       </c>
-      <c r="H104" s="36" t="n">
+      <c r="H106" s="36" t="n">
         <v>16</v>
       </c>
-      <c r="I104" s="36"/>
-      <c r="J104" s="36"/>
-    </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C105" s="25" t="s">
-        <v>142</v>
-      </c>
-      <c r="D105" s="26"/>
-      <c r="E105" s="26"/>
-      <c r="F105" s="26"/>
-      <c r="G105" s="26" t="n">
-        <f aca="false">SUM(G104:G104)</f>
+      <c r="I106" s="36"/>
+      <c r="J106" s="36"/>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C107" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="D107" s="26"/>
+      <c r="E107" s="26"/>
+      <c r="F107" s="26"/>
+      <c r="G107" s="26" t="n">
+        <f aca="false">SUM(G106:G106)</f>
         <v>0</v>
       </c>
-      <c r="H105" s="27" t="n">
-        <f aca="false">SUM(H104:H104)</f>
+      <c r="H107" s="27" t="n">
+        <f aca="false">SUM(H106:H106)</f>
         <v>16</v>
       </c>
-      <c r="I105" s="27"/>
-      <c r="J105" s="27"/>
-    </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C108" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="D108" s="16"/>
-      <c r="E108" s="16"/>
-      <c r="F108" s="16"/>
-      <c r="G108" s="16"/>
-      <c r="H108" s="16"/>
-      <c r="I108" s="16"/>
-      <c r="J108" s="16"/>
-    </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C109" s="19" t="s">
+      <c r="I107" s="27"/>
+      <c r="J107" s="27"/>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C110" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="D109" s="20"/>
-      <c r="E109" s="20"/>
-      <c r="F109" s="20"/>
-      <c r="G109" s="20"/>
-      <c r="H109" s="22" t="n">
-        <f aca="false">H99</f>
-        <v>31</v>
-      </c>
-      <c r="I109" s="22"/>
-      <c r="J109" s="22"/>
-    </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C110" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="D110" s="20"/>
-      <c r="E110" s="20"/>
-      <c r="F110" s="20"/>
-      <c r="G110" s="20"/>
-      <c r="H110" s="22" t="n">
-        <f aca="false">H105</f>
-        <v>16</v>
-      </c>
-      <c r="I110" s="22"/>
-      <c r="J110" s="22"/>
+      <c r="D110" s="16"/>
+      <c r="E110" s="16"/>
+      <c r="F110" s="16"/>
+      <c r="G110" s="16"/>
+      <c r="H110" s="16"/>
+      <c r="I110" s="16"/>
+      <c r="J110" s="16"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C111" s="19" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D111" s="20"/>
       <c r="E111" s="20"/>
       <c r="F111" s="20"/>
       <c r="G111" s="20"/>
-      <c r="H111" s="36" t="n">
+      <c r="H111" s="22" t="n">
+        <f aca="false">H101</f>
+        <v>31</v>
+      </c>
+      <c r="I111" s="22"/>
+      <c r="J111" s="22"/>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C112" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="D112" s="20"/>
+      <c r="E112" s="20"/>
+      <c r="F112" s="20"/>
+      <c r="G112" s="20"/>
+      <c r="H112" s="22" t="n">
+        <f aca="false">H107</f>
+        <v>16</v>
+      </c>
+      <c r="I112" s="22"/>
+      <c r="J112" s="22"/>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C113" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="D113" s="20"/>
+      <c r="E113" s="20"/>
+      <c r="F113" s="20"/>
+      <c r="G113" s="20"/>
+      <c r="H113" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="I111" s="36"/>
-      <c r="J111" s="36"/>
-    </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C112" s="29" t="s">
-        <v>149</v>
-      </c>
-      <c r="D112" s="37"/>
-      <c r="E112" s="37"/>
-      <c r="F112" s="37"/>
-      <c r="G112" s="37"/>
-      <c r="H112" s="37" t="n">
-        <f aca="false">SUM(H109:H111)</f>
+      <c r="I113" s="36"/>
+      <c r="J113" s="36"/>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C114" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="D114" s="37"/>
+      <c r="E114" s="37"/>
+      <c r="F114" s="37"/>
+      <c r="G114" s="37"/>
+      <c r="H114" s="37" t="n">
+        <f aca="false">SUM(H111:H113)</f>
         <v>48</v>
       </c>
-      <c r="I112" s="37"/>
-      <c r="J112" s="37"/>
-    </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C115" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="D115" s="16"/>
-      <c r="E115" s="16"/>
-      <c r="F115" s="16"/>
-      <c r="G115" s="16"/>
-      <c r="H115" s="16"/>
-      <c r="I115" s="16"/>
-      <c r="J115" s="16"/>
-    </row>
-    <row r="116" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C116" s="17" t="s">
+      <c r="I114" s="37"/>
+      <c r="J114" s="37"/>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C117" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="D117" s="16"/>
+      <c r="E117" s="16"/>
+      <c r="F117" s="16"/>
+      <c r="G117" s="16"/>
+      <c r="H117" s="16"/>
+      <c r="I117" s="16"/>
+      <c r="J117" s="16"/>
+    </row>
+    <row r="118" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C118" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="D116" s="18" t="s">
+      <c r="D118" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="E116" s="18" t="s">
+      <c r="E118" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F116" s="18" t="s">
+      <c r="F118" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="G116" s="18" t="s">
+      <c r="G118" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H116" s="18" t="s">
+      <c r="H118" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I116" s="18"/>
-      <c r="J116" s="18"/>
-    </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C117" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="D117" s="24" t="n">
-        <f aca="false">2.5+1.75+1.75</f>
-        <v>6</v>
-      </c>
-      <c r="E117" s="24" t="n">
-        <f aca="false">6-D117</f>
-        <v>0</v>
-      </c>
-      <c r="F117" s="20" t="s">
-        <v>129</v>
-      </c>
-      <c r="G117" s="24" t="n">
-        <f aca="false">E117*H117</f>
-        <v>0</v>
-      </c>
-      <c r="H117" s="36" t="n">
-        <v>14</v>
-      </c>
-      <c r="I117" s="36"/>
-      <c r="J117" s="36"/>
-    </row>
-    <row r="118" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C118" s="19" t="s">
-        <v>151</v>
-      </c>
-      <c r="D118" s="24" t="n">
-        <f aca="false">2.6+2.2</f>
-        <v>4.8</v>
-      </c>
-      <c r="E118" s="24" t="n">
-        <f aca="false">6-D118</f>
-        <v>1.2</v>
-      </c>
-      <c r="F118" s="20" t="s">
-        <v>152</v>
-      </c>
-      <c r="G118" s="24" t="n">
-        <f aca="false">E118*H118</f>
-        <v>18</v>
-      </c>
-      <c r="H118" s="36" t="n">
-        <v>15</v>
-      </c>
-      <c r="I118" s="36"/>
-      <c r="J118" s="36"/>
+      <c r="I118" s="18"/>
+      <c r="J118" s="18"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C119" s="19" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="D119" s="24" t="n">
-        <f aca="false">2.1+2.1+1.8</f>
+        <f aca="false">2.5+1.75+1.75</f>
         <v>6</v>
       </c>
       <c r="E119" s="24" t="n">
@@ -3721,146 +3724,221 @@
         <v>0</v>
       </c>
       <c r="H119" s="36" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I119" s="36"/>
       <c r="J119" s="36"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C120" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="D120" s="24" t="n">
+        <f aca="false">2.5+1.75+1.75</f>
+        <v>6</v>
+      </c>
+      <c r="E120" s="24" t="n">
+        <f aca="false">6-D120</f>
+        <v>0</v>
+      </c>
+      <c r="F120" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="G120" s="24" t="n">
+        <f aca="false">E120*H120</f>
+        <v>0</v>
+      </c>
+      <c r="H120" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="I120" s="36"/>
+      <c r="J120" s="36"/>
+    </row>
+    <row r="121" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C121" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="D121" s="24" t="n">
+        <f aca="false">2.6+2.2</f>
+        <v>4.8</v>
+      </c>
+      <c r="E121" s="24" t="n">
+        <f aca="false">6-D121</f>
+        <v>1.2</v>
+      </c>
+      <c r="F121" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="G121" s="24" t="n">
+        <f aca="false">E121*H121</f>
+        <v>18</v>
+      </c>
+      <c r="H121" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="I121" s="36"/>
+      <c r="J121" s="36"/>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C122" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="D120" s="24" t="n">
+      <c r="D122" s="24" t="n">
+        <f aca="false">2.1+2.1+1.8</f>
+        <v>6</v>
+      </c>
+      <c r="E122" s="24" t="n">
+        <f aca="false">6-D122</f>
+        <v>0</v>
+      </c>
+      <c r="F122" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="G122" s="24" t="n">
+        <f aca="false">E122*H122</f>
+        <v>0</v>
+      </c>
+      <c r="H122" s="36" t="n">
+        <v>7</v>
+      </c>
+      <c r="I122" s="36"/>
+      <c r="J122" s="36"/>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C123" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="D123" s="24" t="n">
         <f aca="false">2.2+1.8+1.8</f>
         <v>5.8</v>
       </c>
-      <c r="E120" s="24" t="n">
-        <f aca="false">6-D120</f>
+      <c r="E123" s="24" t="n">
+        <f aca="false">6-D123</f>
         <v>0.2</v>
       </c>
-      <c r="F120" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="G120" s="24" t="n">
-        <f aca="false">E120*H120</f>
+      <c r="F123" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="G123" s="24" t="n">
+        <f aca="false">E123*H123</f>
         <v>0.800000000000001</v>
       </c>
-      <c r="H120" s="36" t="n">
+      <c r="H123" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="I120" s="36"/>
-      <c r="J120" s="36"/>
-    </row>
-    <row r="121" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C121" s="19" t="s">
-        <v>155</v>
-      </c>
-      <c r="D121" s="24" t="n">
+      <c r="I123" s="36"/>
+      <c r="J123" s="36"/>
+    </row>
+    <row r="124" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C124" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="D124" s="24" t="n">
         <f aca="false">2.6+1.75</f>
         <v>4.35</v>
       </c>
-      <c r="E121" s="24" t="n">
-        <f aca="false">6-D121</f>
+      <c r="E124" s="24" t="n">
+        <f aca="false">6-D124</f>
         <v>1.65</v>
       </c>
-      <c r="F121" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="G121" s="24" t="n">
-        <f aca="false">E121*H121</f>
+      <c r="F124" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="G124" s="24" t="n">
+        <f aca="false">E124*H124</f>
         <v>4.95</v>
       </c>
-      <c r="H121" s="36" t="n">
+      <c r="H124" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="I121" s="36"/>
-      <c r="J121" s="36"/>
-    </row>
-    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C122" s="19" t="s">
-        <v>156</v>
-      </c>
-      <c r="D122" s="24" t="n">
+      <c r="I124" s="36"/>
+      <c r="J124" s="36"/>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C125" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="D125" s="24" t="n">
         <f aca="false">2.2+1.8+1.75</f>
         <v>5.75</v>
       </c>
-      <c r="E122" s="24" t="n">
-        <f aca="false">6-D122</f>
+      <c r="E125" s="24" t="n">
+        <f aca="false">6-D125</f>
         <v>0.25</v>
       </c>
-      <c r="F122" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="G122" s="24" t="n">
-        <f aca="false">E122*H122</f>
+      <c r="F125" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="G125" s="24" t="n">
+        <f aca="false">E125*H125</f>
         <v>0.25</v>
       </c>
-      <c r="H122" s="36" t="n">
+      <c r="H125" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="I122" s="36"/>
-      <c r="J122" s="36"/>
-    </row>
-    <row r="123" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C123" s="19" t="s">
-        <v>157</v>
-      </c>
-      <c r="D123" s="24" t="n">
+      <c r="I125" s="36"/>
+      <c r="J125" s="36"/>
+    </row>
+    <row r="126" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C126" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="D126" s="24" t="n">
         <f aca="false">2.2+2.2</f>
         <v>4.4</v>
       </c>
-      <c r="E123" s="24" t="n">
-        <f aca="false">6-D123</f>
+      <c r="E126" s="24" t="n">
+        <f aca="false">6-D126</f>
         <v>1.6</v>
       </c>
-      <c r="F123" s="20" t="s">
-        <v>139</v>
-      </c>
-      <c r="G123" s="24" t="n">
-        <f aca="false">E123*H123</f>
+      <c r="F126" s="20" t="s">
+        <v>140</v>
+      </c>
+      <c r="G126" s="24" t="n">
+        <f aca="false">E126*H126</f>
         <v>1.6</v>
       </c>
-      <c r="H123" s="36" t="n">
+      <c r="H126" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="I123" s="36"/>
-      <c r="J123" s="36"/>
-    </row>
-    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C124" s="25" t="s">
-        <v>142</v>
-      </c>
-      <c r="D124" s="26"/>
-      <c r="E124" s="26"/>
-      <c r="F124" s="26"/>
-      <c r="G124" s="26" t="n">
-        <f aca="false">SUM(G117:G123)</f>
+      <c r="I126" s="36"/>
+      <c r="J126" s="36"/>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C127" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="D127" s="26"/>
+      <c r="E127" s="26"/>
+      <c r="F127" s="26"/>
+      <c r="G127" s="26" t="n">
+        <f aca="false">SUM(G119:G126)</f>
         <v>25.6</v>
       </c>
-      <c r="H124" s="27" t="n">
-        <f aca="false">SUM(H117:H123)</f>
+      <c r="H127" s="27" t="n">
+        <f aca="false">SUM(H119:H126)</f>
         <v>45</v>
       </c>
-      <c r="I124" s="27"/>
-      <c r="J124" s="27"/>
-    </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C126" s="38" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C127" s="38" t="s">
+      <c r="I127" s="27"/>
+      <c r="J127" s="27"/>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C129" s="38" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C128" s="38" t="s">
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C130" s="38" t="s">
         <v>160</v>
       </c>
     </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C131" s="38" t="s">
+        <v>161</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="104">
+  <mergeCells count="107">
     <mergeCell ref="C5:J5"/>
     <mergeCell ref="H6:J6"/>
     <mergeCell ref="H7:J7"/>
@@ -3934,8 +4012,8 @@
     <mergeCell ref="H83:J83"/>
     <mergeCell ref="H84:J84"/>
     <mergeCell ref="H85:J85"/>
-    <mergeCell ref="C88:J88"/>
-    <mergeCell ref="H89:J89"/>
+    <mergeCell ref="H86:J86"/>
+    <mergeCell ref="C89:J89"/>
     <mergeCell ref="H90:J90"/>
     <mergeCell ref="H91:J91"/>
     <mergeCell ref="H92:J92"/>
@@ -3946,18 +4024,18 @@
     <mergeCell ref="H97:J97"/>
     <mergeCell ref="H98:J98"/>
     <mergeCell ref="H99:J99"/>
-    <mergeCell ref="C102:J102"/>
-    <mergeCell ref="H103:J103"/>
-    <mergeCell ref="H104:J104"/>
+    <mergeCell ref="H100:J100"/>
+    <mergeCell ref="H101:J101"/>
+    <mergeCell ref="C104:J104"/>
     <mergeCell ref="H105:J105"/>
-    <mergeCell ref="C108:J108"/>
-    <mergeCell ref="H109:J109"/>
-    <mergeCell ref="H110:J110"/>
+    <mergeCell ref="H106:J106"/>
+    <mergeCell ref="H107:J107"/>
+    <mergeCell ref="C110:J110"/>
     <mergeCell ref="H111:J111"/>
     <mergeCell ref="H112:J112"/>
-    <mergeCell ref="C115:J115"/>
-    <mergeCell ref="H116:J116"/>
-    <mergeCell ref="H117:J117"/>
+    <mergeCell ref="H113:J113"/>
+    <mergeCell ref="H114:J114"/>
+    <mergeCell ref="C117:J117"/>
     <mergeCell ref="H118:J118"/>
     <mergeCell ref="H119:J119"/>
     <mergeCell ref="H120:J120"/>
@@ -3965,6 +4043,9 @@
     <mergeCell ref="H122:J122"/>
     <mergeCell ref="H123:J123"/>
     <mergeCell ref="H124:J124"/>
+    <mergeCell ref="H125:J125"/>
+    <mergeCell ref="H126:J126"/>
+    <mergeCell ref="H127:J127"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3996,49 +4077,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B5" s="39" t="n">
         <v>1</v>
@@ -4069,12 +4150,12 @@
         <v>0.7791</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B6" s="39" t="n">
         <v>2</v>
@@ -4104,12 +4185,12 @@
         <v>0.4914</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B7" s="39" t="n">
         <v>2</v>
@@ -4139,12 +4220,12 @@
         <v>0.6426</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B8" s="39" t="n">
         <v>4</v>
@@ -4174,12 +4255,12 @@
         <v>0.9408</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="43" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B9" s="44"/>
       <c r="C9" s="44"/>
@@ -4196,12 +4277,12 @@
         <v>2.8539</v>
       </c>
       <c r="J9" s="44" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B11" s="39" t="n">
         <v>1</v>
@@ -4231,7 +4312,7 @@
         <v>0.252</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>